<commit_message>
update to trial times
</commit_message>
<xml_diff>
--- a/data/Study_dates_MeLiDos_IZTECH.xlsx
+++ b/data/Study_dates_MeLiDos_IZTECH.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zauner/Documents/Arbeit/12-TUM/WP2.2.5_Data_Analysis/DidikogluEtAl_Dataset_2025/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zauner/Documents/Arbeit/12-TUM/MeLiDos/WP2.2.5_Data_Analysis/DidikogluEtAl_Dataset_2025/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C2B96B-8C13-7F45-B0FD-E122257C4730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933C69BD-6FA2-A84B-A4B5-034FD40FE832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="500" windowWidth="49960" windowHeight="28300" xr2:uid="{EB2C5E3B-016F-4147-BA32-349D8E1D3953}"/>
+    <workbookView xWindow="1540" yWindow="600" windowWidth="49660" windowHeight="28200" xr2:uid="{EB2C5E3B-016F-4147-BA32-349D8E1D3953}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1518,13 +1518,13 @@
         <v>10</v>
       </c>
       <c r="D34" s="5">
-        <v>45733.563194444447</v>
+        <v>45736.563194444447</v>
       </c>
       <c r="E34" s="5">
-        <v>45733.56527777778</v>
+        <v>45736.56527777778</v>
       </c>
       <c r="F34" s="5">
-        <v>45733.576388888891</v>
+        <v>45736.576388888891</v>
       </c>
       <c r="G34" s="5">
         <v>45743.510416666664</v>
@@ -1545,13 +1545,13 @@
         <v>10</v>
       </c>
       <c r="D35" s="5">
-        <v>45733.563194444447</v>
+        <v>45736.563194444447</v>
       </c>
       <c r="E35" s="5">
-        <v>45733.56527777778</v>
+        <v>45736.56527777778</v>
       </c>
       <c r="F35" s="5">
-        <v>45733.576388888891</v>
+        <v>45736.576388888891</v>
       </c>
       <c r="G35" s="5">
         <v>45743.510416666664</v>
@@ -1572,13 +1572,13 @@
         <v>10</v>
       </c>
       <c r="D36" s="5">
-        <v>45733.563194444447</v>
+        <v>45736.563194444447</v>
       </c>
       <c r="E36" s="5">
-        <v>45733.56527777778</v>
+        <v>45736.56527777778</v>
       </c>
       <c r="F36" s="5">
-        <v>45733.576388888891</v>
+        <v>45736.576388888891</v>
       </c>
       <c r="G36" s="5">
         <v>45743.510416666664</v>

</xml_diff>